<commit_message>
feat: gerar modelo oficial MESTRE UNICO com as 9 abas completas GeoRoutePlan.xlsx
</commit_message>
<xml_diff>
--- a/Ficheiros EXCEL/GeoRoutePlan.xlsx
+++ b/Ficheiros EXCEL/GeoRoutePlan.xlsx
@@ -7,11 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Armazém" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Rotas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Motoristas e Carros" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Justificação entregas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Instruções" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Armazéns" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Frota" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Entregas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Regras" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Rotas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Manifestos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Motoristas e Carros" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Justificação entregas" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Instruções" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41,7 +45,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +80,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
         <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B21B6"/>
+        <bgColor rgb="005B21B6"/>
       </patternFill>
     </fill>
     <fill>
@@ -125,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -155,6 +165,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -522,18 +535,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="37" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -582,57 +596,67 @@
           <t>Tempo_Carga_Min</t>
         </is>
       </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Contacto_Responsavel</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Armazém Principal</t>
+          <t>Armazém Lisboa Central</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Estrada 10, Quinta Maçarocas</t>
+          <t>Avenida Severiano Falcão 16A</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>2695-719</t>
+          <t>2685-379</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>São João da Talha</t>
+          <t>Prior Velho</t>
         </is>
       </c>
       <c r="E2" s="6" t="n">
-        <v>38.8245</v>
+        <v>38.7842</v>
       </c>
       <c r="F2" s="6" t="n">
-        <v>-9.091200000000001</v>
+        <v>-9.123799999999999</v>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="I2" s="5" t="n">
-        <v>20</v>
+        <v>30</v>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>912345678</t>
+        </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Pólo Norte (Maia)</t>
+          <t>Armazém Norte Maia</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Rua Manuel Sousa Moreira Cruz 240</t>
+          <t>Rua de Manuel Sousa Moreira Cruz 240</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -658,11 +682,16 @@
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I3" s="8" t="n">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>923456789</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -676,12 +705,590 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Armazem</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Veiculo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Capacidade_KG</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Capacidade_Vol</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Velocidade_Media</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Hora_Inicio_Turno</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Hora_Fim_Turno</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Custo_KM</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Custo_Hora</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Max_Entregas</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Regras</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Motorista_Nome</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>Motorista_Telemovel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Armazém Lisboa Central</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Carrinha Pequena 01</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>800</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I2" s="6" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>[PEQUENO]</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Manuel Silva</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>910000001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Armazém Lisboa Central</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Carrinha Longo Curso 02</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="J3" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>[ALARGADO]</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>António Santos</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>910000002</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="27" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Armazem</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Doc_ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Morada</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>CP</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Localidade</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Telefone_Cliente</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Peso_KG</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Volume_M3</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Janela1_Inicio</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Janela1_Fim</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>Tempo_Descarga_Min</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Regras</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Vendedor</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Valor_Cobrar</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Notas_Entrega</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Armazém Lisboa Central</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>FT 2026/101</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Restaurante Alfama</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Rua de São Tomé 14</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>1100-563</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="n">
+        <v>38.7138</v>
+      </c>
+      <c r="H2" s="6" t="n">
+        <v>-9.130100000000001</v>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>912345670</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="K2" s="6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>[PEQUENO]</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>TNB</t>
+        </is>
+      </c>
+      <c r="Q2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="4" t="inlineStr">
+        <is>
+          <t>Entregar porta cais</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Armazém Lisboa Central</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>FT 2026/102</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Hotel Avenida Palace</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Rua 1º de Dezembro 123</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>1200-359</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>38.715</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>-9.141500000000001</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>912345671</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>320</v>
+      </c>
+      <c r="K3" s="9" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>[ALARGADO]</t>
+        </is>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>TNB</t>
+        </is>
+      </c>
+      <c r="Q3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="7" t="inlineStr">
+        <is>
+          <t>Recepção de mercadorias</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="63" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tag_Veiculo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Permissao</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Tag_Entrega</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Descricao</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>PEQUENO</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>PEQUENO</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Veículo pequeno acede a centros históricos e ruas estreitas</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>ALARGADO</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>NAO</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>PEQUENO</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Veículo de longo curso proibido em ruas estreitas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -693,7 +1300,7 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -907,214 +1514,7 @@
       </c>
       <c r="O3" s="7" t="inlineStr">
         <is>
-          <t>Cais das traseiras</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>D17932331</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Sérgio Azul</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Rua Virgínia Vitorino 10, 7esquerdo</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>1600-784</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Rota Norte 1</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="K4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L4" s="5" t="inlineStr">
-        <is>
-          <t>910000003</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>TNB</t>
-        </is>
-      </c>
-      <c r="N4" s="6" t="n">
-        <v>120.5</v>
-      </c>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>Cobrar no ato de entrega</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>D17931267</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Costa &amp; Associados</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Rua 3, N16 3 C</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Pedrouços</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>1500-605</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>Rota Norte 1</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="J5" s="9" t="n">
-        <v>336</v>
-      </c>
-      <c r="K5" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="L5" s="8" t="inlineStr">
-        <is>
-          <t>910000004</t>
-        </is>
-      </c>
-      <c r="M5" s="8" t="inlineStr">
-        <is>
-          <t>TNB</t>
-        </is>
-      </c>
-      <c r="N5" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="7" t="inlineStr">
-        <is>
-          <t>Ligar antes de chegar</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>D17863817</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Vanessa Machado</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Av. Uruguai Nº 19, 1º Esq.</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>1500-611</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Rota Sul 2</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="n">
-        <v>174</v>
-      </c>
-      <c r="K6" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>910000005</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>TNB</t>
-        </is>
-      </c>
-      <c r="N6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="4" t="inlineStr">
-        <is>
-          <t>Tocar à campainha</t>
+          <t>Cais traseiras</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1523,138 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Armazem</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Veiculo</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Motorista</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>Total_Paragens</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>Volume_Total_M3</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>Peso_Total_KG</t>
+        </is>
+      </c>
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>Taxa_Ocupacao_Peso</t>
+        </is>
+      </c>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
+          <t>Distancia_Total_KM</t>
+        </is>
+      </c>
+      <c r="I1" s="10" t="inlineStr">
+        <is>
+          <t>Tempo_Total_Estimado</t>
+        </is>
+      </c>
+      <c r="J1" s="10" t="inlineStr">
+        <is>
+          <t>Custo_Total_Estimado</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Lista_Documentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Armazém Lisboa Central</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Carrinha Pequena 01</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Manuel Silva</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F2" s="6" t="n">
+        <v>130</v>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>16.2%</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>02h 25m</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>FT 2026/101, FT 2026/104</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1269,7 +1800,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1371,52 +1902,52 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="56" customWidth="1" min="6" max="6"/>
+    <col width="41" customWidth="1" min="5" max="5"/>
+    <col width="61" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Secção</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
-        <is>
-          <t>Campo</t>
-        </is>
-      </c>
-      <c r="C1" s="10" t="inlineStr">
-        <is>
-          <t>Obrigatoriedade</t>
-        </is>
-      </c>
-      <c r="D1" s="10" t="inlineStr">
-        <is>
-          <t>Formato</t>
-        </is>
-      </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Campo_ou_Regra</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Obrigatorio</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Formato_Aceite</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Exemplo</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
-        <is>
-          <t>Descrição / Dica</t>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>Descricao_e_Recomendacoes</t>
         </is>
       </c>
     </row>
@@ -1443,12 +1974,12 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Campos essenciais para geocodificação e rotas.</t>
+          <t>Ex: Nome_Armazem, Morada, CP</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Se faltar, o sistema não consegue calcular.</t>
+          <t>Campos essenciais para geocodificação e cálculo de rotas.</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1991,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Azul Claro (#2563EB)</t>
+          <t>Azul Mais Claro (#2563EB)</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -1475,12 +2006,12 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Janelas, Contactos, Pesos, Volumes.</t>
+          <t>Ex: Janelas, Custos, Capacidade</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Aumenta a precisão de cálculo e relatórios.</t>
+          <t>Aumenta a precisão de cálculo de tempos e indicadores.</t>
         </is>
       </c>
     </row>
@@ -1492,7 +2023,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Cinza (#64748B)</t>
+          <t>Cinza Ardósia (#64748B)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -1507,29 +2038,29 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Notas, Vendedor, Valor a Cobrar.</t>
+          <t>Ex: Localidade, Notas, Valor a Cobrar</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Informação adicional de suporte.</t>
+          <t>Informação complementar.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>1. Armazém</t>
+          <t>1. Armazéns</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Morada &amp; CP</t>
+          <t>Nome_Armazem &amp; CP</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -1539,93 +2070,93 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>2695-719</t>
+          <t>Armazém Central / 2685-379</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Ponto de partida e chegada das carrinhas.</t>
+          <t>Identificador e morada do polo logístico.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2. Rotas</t>
+          <t>2. Frota</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Cliente, Morada, CP</t>
+          <t>Veiculo &amp; Capacidade_KG</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Texto / XXXX-XXX</t>
+          <t>Texto / Decimal</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>1750-168 Lisboa</t>
+          <t>Carrinha 01 / 800</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Dados dos destinatários.</t>
+          <t>Viaturas e capacidades para otimização.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>3. Motoristas</t>
+          <t>3. Entregas</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Motorista &amp; PIN</t>
+          <t>Cliente, Morada, CP, Janelas</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Texto / 4 dígitos</t>
+          <t>Texto / HH:MM</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>1111</t>
+          <t>FT 2026/101 / 09:00 - 13:00</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Código para o motorista entrar na rota na App móvel.</t>
+          <t>Paragens a visitar.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>4. Justificações</t>
+          <t>4. Regras</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Motivos de Falha</t>
+          <t>Tag_Veiculo &amp; Tag_Entrega</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1635,12 +2166,140 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Cliente Fechado</t>
+          <t>PEQUENO / SIM / PEQUENO</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Opções que aparecem no telemóvel do motorista.</t>
+          <t>Restrições de acesso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>5. Rotas</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Rotas Calculadas</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Leitura</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Ordem &amp; Janelas</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Rota Norte 1 (#1)</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Sequência otimizada de entrega.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>6. Manifestos</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Resumo de Carga</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Leitura</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Totais KM / Custo</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Total 27.7 km</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Folha de carga para motorista.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>7. Motoristas e Carros</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Motorista &amp; PIN</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Texto / 4 dígitos</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>João Silva / 1111</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Credenciais de acesso à WebApp móvel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>8. Justificação</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Motivo de Falha</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Cliente Ausente / Fechado</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Opções predefinidas de não entrega.</t>
         </is>
       </c>
     </row>

</xml_diff>